<commit_message>
Added Sheet 2 for Order list
</commit_message>
<xml_diff>
--- a/Accelerometer Parts List.xlsx
+++ b/Accelerometer Parts List.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlguy\New Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413603B5-E080-4E3A-B4B6-93CAD2686039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D82D00-9963-4119-97A4-488CA5ADF99F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="First Accelerometer PCB Order" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="120">
   <si>
     <t>Part Description</t>
   </si>
@@ -336,14 +337,75 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/yageo/RC0805FR-07100KL/727544</t>
+  </si>
+  <si>
+    <t>need to figure out wire gauge we are using</t>
+  </si>
+  <si>
+    <t>OshPark</t>
+  </si>
+  <si>
+    <t>OshStencil</t>
+  </si>
+  <si>
+    <t>Notes: For first order, we already have the swan, the clock, the accelerometer, the batteries, an OLED screen, and plenty of buttons</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/jst-sales-america-inc/SPH-002T-P0-5S/26216268</t>
+  </si>
+  <si>
+    <t>455-1127-100-ND</t>
+  </si>
+  <si>
+    <t>SPH-002T-P0.5S</t>
+  </si>
+  <si>
+    <t>CONN SOCKET 24-30AWG CRIMP TIN</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/cnc-tech/1007-24-1-2000-001-1-TS/28220524</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/cnc-tech/1007-24-1-2000-004-1-TS/28220605</t>
+  </si>
+  <si>
+    <t>Paste Stencil</t>
+  </si>
+  <si>
+    <t>https://oshpark.com/shared_projects/LVQwHZoq</t>
+  </si>
+  <si>
+    <t>CNC Tech</t>
+  </si>
+  <si>
+    <t>1175-1007-24-1-2000-004-1-TS-ND</t>
+  </si>
+  <si>
+    <t>1007-24-1-2000-004-1-TS</t>
+  </si>
+  <si>
+    <t>WIRE 24AWG RED STRAND FEET</t>
+  </si>
+  <si>
+    <t>1175-1007-24-1-2000-001-1-TS-ND</t>
+  </si>
+  <si>
+    <t>WIRE 24AWG BLK STRAND FEET</t>
+  </si>
+  <si>
+    <t>1007-24-1-2000-001-1-TS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000_);[Red]\(&quot;$&quot;#,##0.0000\)"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -411,7 +473,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -420,6 +482,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="8" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -735,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="39.26953125" customWidth="1"/>
@@ -968,7 +1032,7 @@
         <f>E7*F7</f>
         <v>0.1</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="4" t="s">
         <v>76</v>
       </c>
       <c r="J7" t="s">
@@ -1320,6 +1384,11 @@
       <c r="G23" s="3">
         <f>G20+G22</f>
         <v>54.739999999999995</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1331,8 +1400,441 @@
     <hyperlink ref="H22" r:id="rId5" xr:uid="{F00F8E76-9440-41F1-9983-F88FE3FF92F9}"/>
     <hyperlink ref="H6" r:id="rId6" location="technical-details" xr:uid="{2DF40FBC-FC77-4FBB-927F-4F592874E487}"/>
     <hyperlink ref="H12" r:id="rId7" xr:uid="{4611F87B-6738-49CF-BABA-7107C1E2B1D5}"/>
+    <hyperlink ref="I7" r:id="rId8" xr:uid="{6C75CCA2-2FCB-44F0-BAA5-0079A3856A71}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE43E244-E934-476D-A364-71F29400FAE1}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" customWidth="1"/>
+    <col min="3" max="3" width="16.36328125" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" customWidth="1"/>
+    <col min="6" max="6" width="9.6328125" customWidth="1"/>
+    <col min="7" max="8" width="14.1796875" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2" s="8">
+        <v>0.49</v>
+      </c>
+      <c r="G2" s="3">
+        <f t="shared" ref="G2" si="0">E2*F2</f>
+        <v>1.47</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" s="5"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="G3" s="3">
+        <f>E3*F3</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4" s="8">
+        <v>4.0899999999999999E-2</v>
+      </c>
+      <c r="G4" s="3">
+        <f t="shared" ref="G4:G10" si="1">E4*F4</f>
+        <v>4.09</v>
+      </c>
+      <c r="H4" t="s">
+        <v>105</v>
+      </c>
+      <c r="J4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.49</v>
+      </c>
+      <c r="G5" s="3">
+        <f t="shared" si="1"/>
+        <v>1.47</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6" s="8">
+        <v>0.61</v>
+      </c>
+      <c r="G6" s="3">
+        <f t="shared" si="1"/>
+        <v>1.83</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="6">
+        <v>20</v>
+      </c>
+      <c r="F7" s="9">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="G7" s="3">
+        <f t="shared" si="1"/>
+        <v>0.68</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="G8" s="3">
+        <f t="shared" si="1"/>
+        <v>1.9500000000000002</v>
+      </c>
+      <c r="H8" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9" s="8">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="G9" s="3">
+        <f t="shared" si="1"/>
+        <v>0.34</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="I9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10">
+        <v>5033981892</v>
+      </c>
+      <c r="D10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10" s="3">
+        <v>2.62</v>
+      </c>
+      <c r="G10" s="3">
+        <f>E10*F10</f>
+        <v>7.86</v>
+      </c>
+      <c r="H10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E11">
+        <v>10</v>
+      </c>
+      <c r="F11" s="8">
+        <v>0.439</v>
+      </c>
+      <c r="G11" s="3">
+        <f t="shared" ref="G11:G12" si="2">E11*F11</f>
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="H11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0.439</v>
+      </c>
+      <c r="G12" s="3">
+        <f t="shared" si="2"/>
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="H12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>32.950000000000003</v>
+      </c>
+      <c r="G14" s="3">
+        <f t="shared" ref="G13:G14" si="3">E14*F14</f>
+        <v>32.950000000000003</v>
+      </c>
+      <c r="H14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F17" t="s">
+        <v>104</v>
+      </c>
+      <c r="G17" s="3">
+        <f>SUM(G2:G14)</f>
+        <v>61.72</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{C0FAAA57-36CF-4FD4-B1C5-2E553F7E135C}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{BB6A0EF0-CA79-4DA5-BC3B-A25585134DD4}"/>
+    <hyperlink ref="I2" r:id="rId3" xr:uid="{019A236E-D2DB-4CB1-90AB-7CF61FEC7D33}"/>
+    <hyperlink ref="H3" r:id="rId4" xr:uid="{CF106BCC-1B59-40D2-84C6-969F8BAEA402}"/>
+    <hyperlink ref="H7" r:id="rId5" xr:uid="{E4B1C75A-C253-4D42-AA8F-162D4E4EB9F6}"/>
+    <hyperlink ref="H5" r:id="rId6" xr:uid="{A381883F-7E88-486C-84C5-7002F7CBB814}"/>
+    <hyperlink ref="H6" r:id="rId7" xr:uid="{B38C5576-E2C0-47C0-8454-B5FAB3F28022}"/>
+    <hyperlink ref="H9" r:id="rId8" xr:uid="{E6937922-3549-4B98-A42F-FAA02C8572BF}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>